<commit_message>
feat(F-NAR-016): TREE-DIF-027 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-027.xlsx
+++ b/stories/arbres/TREE-DIF-027.xlsx
@@ -1383,12 +1383,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Le panier reste ouvert, près des pieds. La cuillère, la clochette, et la ficelle. Tu prends quoi d'abord, Sarah ?</t>
+          <t>Le panier reste ouvert, près des pieds. Une cuillère y brille, encore tiède. Une clochette, puis une ficelle, à côté. Tu prends quoi d'abord, Sarah ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le panier reste ouvert, près des pieds. La cuillère, la clochette, et la ficelle. Tu prends quoi d'abord, Sarah ?</t>
+          <t>Le panier reste ouvert, près des pieds. Une cuillère y brille, encore tiède. Une clochette, puis une ficelle, à côté. Tu prends quoi d'abord, Sarah ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1548,7 +1548,8 @@
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Le panier reste ouvert, près des pieds.
-narrateur|La cuillère, la clochette, et la ficelle.
+narrateur|Une cuillère y brille, encore tiède.
+narrateur|Une clochette, puis une ficelle, à côté.
 papa|Tu prends quoi d'abord, Sarah ?</t>
         </is>
       </c>
@@ -1576,12 +1577,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord la cuillère chaude. Elle sent le savon. Le métal est encore un peu mouillé. Elle la tend vers Aniss, tout près. Dis ding ! Aniss pose un doigt sur le creux. Ça fait un tout petit tic. La clochette et la ficelle viennent aussi. Papa glisse le tout dans le panier. Les trois affaires restent ensemble. Aniss, on part ? Aniss hoche la tête, tout petit. La cuillère d'abord, vous l'avez.</t>
+          <t>Sarah prend d'abord la cuillère chaude. Elle sent le savon. Le métal est encore un peu mouillé. Elle la tend vers Aniss, tout près. Dis ding ! Aniss pose un doigt sur le creux. Ça fait un tout petit tic. La clochette et la ficelle viennent aussi. Papa glisse le tout dans le panier. Rien ne reste sur la table. Aniss, on part ? Aniss hoche la tête, tout petit. La cuillère d'abord, vous l'avez.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord la cuillère chaude. Elle sent le savon. Le métal est encore un peu mouillé. Elle la tend vers Aniss, tout près. Dis ding ! Aniss pose un doigt sur le creux. Ça fait un tout petit tic. La clochette et la ficelle viennent aussi. Papa glisse le tout dans le panier. Les trois affaires restent ensemble. Aniss, on part ? Aniss hoche la tête, tout petit. La cuillère d'abord, vous l'avez.</t>
+          <t>Sarah prend d'abord la cuillère chaude. Elle sent le savon. Le métal est encore un peu mouillé. Elle la tend vers Aniss, tout près. Dis ding ! Aniss pose un doigt sur le creux. Ça fait un tout petit tic. La clochette et la ficelle viennent aussi. Papa glisse le tout dans le panier. Rien ne reste sur la table. Aniss, on part ? Aniss hoche la tête, tout petit. La cuillère d'abord, vous l'avez.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1725,7 +1726,7 @@
 narrateur|Ça fait un tout petit tic.
 maman|La clochette et la ficelle viennent aussi.
 narrateur|Papa glisse le tout dans le panier.
-narrateur|Les trois affaires restent ensemble.
+narrateur|Rien ne reste sur la table.
 enfant-f|Aniss, on part ?
 narrateur|Aniss hoche la tête, tout petit.
 papa|La cuillère d'abord, vous l'avez.</t>
@@ -2116,12 +2117,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>La cuillère voyage déjà dans le panier. Sous l'étendoir, un linge pend, encore mouillé. Sur la poutre, un clou brille, trop haut. Sur la marche, le vent pousse déjà. On commence où, pour le fil ?</t>
+          <t>La cuillère voyage déjà dans le panier. Dehors, le fil peut aller en trois coins. Un linge mouillé barre encore l'étendoir. Plus haut, un clou attend sur la poutre. Plus bas, le vent pousse la marche. On commence où, pour le fil ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>La cuillère voyage déjà dans le panier. Sous l'étendoir, un linge pend, encore mouillé. Sur la poutre, un clou brille, trop haut. Sur la marche, le vent pousse déjà. On commence où, pour le fil ?</t>
+          <t>La cuillère voyage déjà dans le panier. Dehors, le fil peut aller en trois coins. Un linge mouillé barre encore l'étendoir. Plus haut, un clou attend sur la poutre. Plus bas, le vent pousse la marche. On commence où, pour le fil ?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2281,9 +2282,10 @@
       <c r="AW7" t="inlineStr">
         <is>
           <t>narrateur|La cuillère voyage déjà dans le panier.
-narrateur|Sous l'étendoir, un linge pend, encore mouillé.
-narrateur|Sur la poutre, un clou brille, trop haut.
-narrateur|Sur la marche, le vent pousse déjà.
+narrateur|Dehors, le fil peut aller en trois coins.
+narrateur|Un linge mouillé barre encore l'étendoir.
+narrateur|Plus haut, un clou attend sur la poutre.
+narrateur|Plus bas, le vent pousse la marche.
 papa|On commence où, pour le fil ?</t>
         </is>
       </c>
@@ -3028,12 +3030,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la cuillère. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge. La cuillère reste un instant sur le bois.</t>
+          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la cuillère. La cuillère attend près du bois, déjà. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la cuillère. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge. La cuillère reste un instant sur le bois.</t>
+          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la cuillère. La cuillère attend près du bois, déjà. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3171,11 +3173,11 @@
           <t>enfant-f|Pour toi.
 narrateur|Sarah tend la cuillère vers Aniss.
 narrateur|Aniss lève le torchon avec la cuillère.
+narrateur|La cuillère attend près du bois, déjà.
 narrateur|Le bois redevient libre, tout doux.
 enfant-f|Il passe !
 maman|Le fil a pris le bord, tout seul.
-papa|Le métal a trouvé le linge.
-narrateur|La cuillère reste un instant sur le bois.</t>
+papa|Le métal a trouvé le linge.</t>
         </is>
       </c>
     </row>
@@ -6547,12 +6549,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord la clochette froide. Elle va tinter. Le métal est un peu rêche. Elle la tend vers Aniss. Dis ding ! Aniss la tient à deux mains. Ça tinte une fois, puis s'arrête. La cuillère et la ficelle viennent aussi. Maman les pose près du panier. Les trois affaires restent ensemble. Aniss, tu viens ? Aniss lève la clochette, tout bas. La clochette d'abord, vous l'avez.</t>
+          <t>Sarah prend d'abord la clochette froide. Elle va tinter. Le métal est un peu rêche. Elle la tend vers Aniss. Dis ding ! Aniss la tient à deux mains. Ça tinte une fois, puis s'arrête. La cuillère et la ficelle viennent aussi. Maman les pose près du panier. Tout part ensemble, déjà. Aniss, tu viens ? Aniss lève la clochette, tout bas. La clochette d'abord, vous l'avez.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord la clochette froide. Elle va tinter. Le métal est un peu rêche. Elle la tend vers Aniss. Dis ding ! Aniss la tient à deux mains. Ça tinte une fois, puis s'arrête. La cuillère et la ficelle viennent aussi. Maman les pose près du panier. Les trois affaires restent ensemble. Aniss, tu viens ? Aniss lève la clochette, tout bas. La clochette d'abord, vous l'avez.</t>
+          <t>Sarah prend d'abord la clochette froide. Elle va tinter. Le métal est un peu rêche. Elle la tend vers Aniss. Dis ding ! Aniss la tient à deux mains. Ça tinte une fois, puis s'arrête. La cuillère et la ficelle viennent aussi. Maman les pose près du panier. Tout part ensemble, déjà. Aniss, tu viens ? Aniss lève la clochette, tout bas. La clochette d'abord, vous l'avez.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -6696,7 +6698,7 @@
 narrateur|Ça tinte une fois, puis s'arrête.
 papa|La cuillère et la ficelle viennent aussi.
 narrateur|Maman les pose près du panier.
-narrateur|Les trois affaires restent ensemble.
+narrateur|Tout part ensemble, déjà.
 enfant-f|Aniss, tu viens ?
 narrateur|Aniss lève la clochette, tout bas.
 maman|La clochette d'abord, vous l'avez.</t>
@@ -7087,12 +7089,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>La clochette voyage déjà dans le panier. Sous l'étendoir, un linge pend, encore mouillé. Sur la poutre, un clou brille, trop haut. Sur la marche, le vent pousse déjà. On commence où, pour le fil ?</t>
+          <t>La clochette voyage déjà dans le panier. Dehors, le fil peut aller en trois coins. Un linge mouillé barre encore l'étendoir. Plus haut, un clou attend sur la poutre. Plus bas, le vent pousse la marche. On commence où, pour le fil ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>La clochette voyage déjà dans le panier. Sous l'étendoir, un linge pend, encore mouillé. Sur la poutre, un clou brille, trop haut. Sur la marche, le vent pousse déjà. On commence où, pour le fil ?</t>
+          <t>La clochette voyage déjà dans le panier. Dehors, le fil peut aller en trois coins. Un linge mouillé barre encore l'étendoir. Plus haut, un clou attend sur la poutre. Plus bas, le vent pousse la marche. On commence où, pour le fil ?</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -7252,9 +7254,10 @@
       <c r="AW35" t="inlineStr">
         <is>
           <t>narrateur|La clochette voyage déjà dans le panier.
-narrateur|Sous l'étendoir, un linge pend, encore mouillé.
-narrateur|Sur la poutre, un clou brille, trop haut.
-narrateur|Sur la marche, le vent pousse déjà.
+narrateur|Dehors, le fil peut aller en trois coins.
+narrateur|Un linge mouillé barre encore l'étendoir.
+narrateur|Plus haut, un clou attend sur la poutre.
+narrateur|Plus bas, le vent pousse la marche.
 papa|On commence où, pour le fil ?</t>
         </is>
       </c>
@@ -7999,12 +8002,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la clochette. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge. La clochette reste un instant sur le bois.</t>
+          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la cuillère. La clochette attend près du bois, déjà. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la clochette. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge. La clochette reste un instant sur le bois.</t>
+          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la cuillère. La clochette attend près du bois, déjà. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8141,12 +8144,12 @@
         <is>
           <t>enfant-f|Pour toi.
 narrateur|Sarah tend la cuillère vers Aniss.
-narrateur|Aniss lève le torchon avec la clochette.
+narrateur|Aniss lève le torchon avec la cuillère.
+narrateur|La clochette attend près du bois, déjà.
 narrateur|Le bois redevient libre, tout doux.
 enfant-f|Il passe !
 maman|Le fil a pris le bord, tout seul.
-papa|Le métal a trouvé le linge.
-narrateur|La clochette reste un instant sur le bois.</t>
+papa|Le métal a trouvé le linge.</t>
         </is>
       </c>
     </row>
@@ -11518,12 +11521,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord la ficelle douce. C'est pour le fil. Elle sent encore le tiroir. Elle tend le peloton vers Aniss. Dis fil ! Aniss enroule un bout, tout lent. Le fil se fait, sans un mot. La cuillère et la clochette viennent aussi. Papa les glisse près du sac. Les trois affaires restent ensemble. Aniss, c'est bon ? Aniss appuie sur le fil, tout calme. La ficelle d'abord, elle tient.</t>
+          <t>Sarah prend d'abord la ficelle douce. C'est pour le fil. Elle sent encore le tiroir. Elle tend le peloton vers Aniss. Dis fil ! Aniss enroule un bout, tout lent. Le fil se fait, sans un mot. La cuillère et la clochette viennent aussi. Papa les glisse près du sac. Le panier les garde, toutes les trois. Aniss, c'est bon ? Aniss appuie sur le fil, tout calme. La ficelle d'abord, elle tient.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord la ficelle douce. C'est pour le fil. Elle sent encore le tiroir. Elle tend le peloton vers Aniss. Dis fil ! Aniss enroule un bout, tout lent. Le fil se fait, sans un mot. La cuillère et la clochette viennent aussi. Papa les glisse près du sac. Les trois affaires restent ensemble. Aniss, c'est bon ? Aniss appuie sur le fil, tout calme. La ficelle d'abord, elle tient.</t>
+          <t>Sarah prend d'abord la ficelle douce. C'est pour le fil. Elle sent encore le tiroir. Elle tend le peloton vers Aniss. Dis fil ! Aniss enroule un bout, tout lent. Le fil se fait, sans un mot. La cuillère et la clochette viennent aussi. Papa les glisse près du sac. Le panier les garde, toutes les trois. Aniss, c'est bon ? Aniss appuie sur le fil, tout calme. La ficelle d'abord, elle tient.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -11667,7 +11670,7 @@
 narrateur|Le fil se fait, sans un mot.
 maman|La cuillère et la clochette viennent aussi.
 narrateur|Papa les glisse près du sac.
-narrateur|Les trois affaires restent ensemble.
+narrateur|Le panier les garde, toutes les trois.
 enfant-f|Aniss, c'est bon ?
 narrateur|Aniss appuie sur le fil, tout calme.
 papa|La ficelle d'abord, elle tient.</t>
@@ -12058,12 +12061,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>La ficelle voyage déjà dans le panier. Sous l'étendoir, un linge pend, encore mouillé. Sur la poutre, un clou brille, trop haut. Sur la marche, le vent pousse déjà. On commence où, pour le fil ?</t>
+          <t>La ficelle voyage déjà dans le panier. Dehors, le fil peut aller en trois coins. Un linge mouillé barre encore l'étendoir. Plus haut, un clou attend sur la poutre. Plus bas, le vent pousse la marche. On commence où, pour le fil ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>La ficelle voyage déjà dans le panier. Sous l'étendoir, un linge pend, encore mouillé. Sur la poutre, un clou brille, trop haut. Sur la marche, le vent pousse déjà. On commence où, pour le fil ?</t>
+          <t>La ficelle voyage déjà dans le panier. Dehors, le fil peut aller en trois coins. Un linge mouillé barre encore l'étendoir. Plus haut, un clou attend sur la poutre. Plus bas, le vent pousse la marche. On commence où, pour le fil ?</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -12223,9 +12226,10 @@
       <c r="AW63" t="inlineStr">
         <is>
           <t>narrateur|La ficelle voyage déjà dans le panier.
-narrateur|Sous l'étendoir, un linge pend, encore mouillé.
-narrateur|Sur la poutre, un clou brille, trop haut.
-narrateur|Sur la marche, le vent pousse déjà.
+narrateur|Dehors, le fil peut aller en trois coins.
+narrateur|Un linge mouillé barre encore l'étendoir.
+narrateur|Plus haut, un clou attend sur la poutre.
+narrateur|Plus bas, le vent pousse la marche.
 papa|On commence où, pour le fil ?</t>
         </is>
       </c>
@@ -12970,12 +12974,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la ficelle. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge. La ficelle reste un instant sur le bois.</t>
+          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la cuillère. La ficelle attend près du bois, déjà. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la ficelle. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge. La ficelle reste un instant sur le bois.</t>
+          <t>Pour toi. Sarah tend la cuillère vers Aniss. Aniss lève le torchon avec la cuillère. La ficelle attend près du bois, déjà. Le bois redevient libre, tout doux. Il passe ! Le fil a pris le bord, tout seul. Le métal a trouvé le linge.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13112,12 +13116,12 @@
         <is>
           <t>enfant-f|Pour toi.
 narrateur|Sarah tend la cuillère vers Aniss.
-narrateur|Aniss lève le torchon avec la ficelle.
+narrateur|Aniss lève le torchon avec la cuillère.
+narrateur|La ficelle attend près du bois, déjà.
 narrateur|Le bois redevient libre, tout doux.
 enfant-f|Il passe !
 maman|Le fil a pris le bord, tout seul.
-papa|Le métal a trouvé le linge.
-narrateur|La ficelle reste un instant sur le bois.</t>
+papa|Le métal a trouvé le linge.</t>
         </is>
       </c>
     </row>
@@ -16483,7 +16487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16526,6 +16530,13 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>